<commit_message>
docs(0916): retract every MFU figure -- the denominator was an A100
torchtitan's get_peak_flops() ends in 'else: assume A100, return 312e12' for any device_name
it does not recognise, and this box reports 'AMD Radeon Graphics' (there is no lspci in the
container either). So every MFU this campaign has printed used an A100 denominator. Today's
run makes it obvious -- it reported 215.63%, which is simply 672.76 / 312.

The tflops column is unaffected; it is FLOPs over time. Corrected across PROGRESS-REPORT.html,
WEEKLY-EN.md and the xlsx attention sheet: the previously reported 'MFU 34% -> 65.4%' now
reads TFLOP/s ~106 -> ~204, and today's run is added at 640.7. Against this campaign's own
measured Triton GEMM roof (1002.7 TF/s at 1100 MHz) that is 63.9%.

The weekly material also gains today's wgrad result: 38,043 tps, 6.21x over unpatched.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
+++ b/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
@@ -18444,7 +18444,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">MFU</t>
+          <t xml:space="preserve">tflop/s (measured)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">~34%</t>
+          <t xml:space="preserve">~106</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18496,7 +18496,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">+ GEMM layout workaround</t>
+          <t xml:space="preserve">+ dgrad layout fix</t>
         </is>
       </c>
       <c r="B43">
@@ -18504,7 +18504,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">65.4%</t>
+          <t xml:space="preserve">~204</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18716,7 +18716,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cross-check: B0 at full clock also measures torch.mm(NN) at just 112.98 tflop/s against 1190.07 for a naive Triton GEMM (10.5x) — same order as A0's 13x. The missing NN tuning library is not specific to the throttled box.</t>
+          <t xml:space="preserve">DO NOT quote MFU from any torchtitan log on this box: get_peak_flops() falls back to "assume A100" (312 TF/s) for an unrecognised device_name, and this box reports "AMD Radeon Graphics". The tflop/s column is correct; mfu is not. || Cross-check: B0 at full clock also measures torch.mm(NN) at just 112.98 tflop/s against 1190.07 for a naive Triton GEMM (10.5x) — same order as A0's 13x. The missing NN tuning library is not specific to the throttled box.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(0916): add today's wgrad result to the attention sheet
Inserts the 0916 end-to-end row (38,043 tps, 640.7 TF/s, n=6, 6.21x over unpatched) after the
dgrad row, with the note that both operands have to change -- either alone leaves the call on
the bad tile at 60-70 TF/s.

Row numbers below the insertion point were renumbered, cell references inside each row
rewritten to match, and the dimension updated. Other tabs' row counts and gemm-hk's
conditional formatting verified unchanged afterwards.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
+++ b/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
@@ -17040,7 +17040,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.5"/>
@@ -18526,195 +18526,225 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t xml:space="preserve">+ wgrad layout fix (0916)</t>
+        </is>
+      </c>
+      <c r="B44">
+        <v>38043.0</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">640.7</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.97%</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n=6 (excl. first run: 37738, sd 0.09%)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.21x over unpatched, 3.28x over dgrad-only. Both operands must change: A.contiguous() AND B N-major -- either alone stays on the bad tile (60-70 TF/s). Step 861 ms. Peak memory unchanged at 141.00 GiB. 5 consecutive runs, zero card faults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t xml:space="preserve">ASM bwd ON / OFF (no workaround)</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t xml:space="preserve">6110.8 / 6128.1</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t xml:space="preserve">3.88% / 3.91%</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t xml:space="preserve">-0.28%, 0.15x sem — not significant; hence ASM bwd defaults OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[5] A0 — where a step goes (8 layers, step-10 torch profile, 5.2 s step)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">module</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ms</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">share</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">[5] A0 — where a step goes (8 layers, step-10 torch profile, 5.2 s step)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">hipBLASLt GEMM</t>
-        </is>
-      </c>
-      <c r="B48">
-        <v>4877.0</v>
+          <t xml:space="preserve">module</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ms</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">94%</t>
+          <t xml:space="preserve">share</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">4727 ms of it (97%) on MT32x16x32 — the wrong solution</t>
+          <t xml:space="preserve">note</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">attention (fwd+bwd)</t>
+          <t xml:space="preserve">hipBLASLt GEMM</t>
         </is>
       </c>
       <c r="B49">
-        <v>171.0</v>
+        <v>4877.0</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3%</t>
+          <t xml:space="preserve">94%</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">bwd_kernel_causal 138.55 + attn_fwd 32.09</t>
+          <t xml:space="preserve">4727 ms of it (97%) on MT32x16x32 — the wrong solution</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t xml:space="preserve">attention (fwd+bwd)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <v>171.0</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.3%</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bwd_kernel_causal 138.55 + attn_fwd 32.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">everything else</t>
         </is>
       </c>
-      <c r="B50">
+      <c r="B51">
         <v>140.0</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t xml:space="preserve">2.7%</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t xml:space="preserve">elementwise / optimizer / reduce / softmax</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOTES</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clocks differ ~2x between the two machines. Absolute values are NOT comparable across machines; no clock conversion is applied anywhere in this sheet.</t>
+          <t xml:space="preserve">NOTES</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">A0 is VR-throttled: rocm-smi reports 1100 MHz, a sysfs sample under sustained load read 943 MHz. Its Hardware MFU column is therefore not a measure of efficiency.</t>
+          <t xml:space="preserve">Clocks differ ~2x between the two machines. Absolute values are NOT comparable across machines; no clock conversion is applied anywhere in this sheet.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every value re-derived from the raw ledgers. Where a published document disagreed, the ledger wins and the note says so. See LEDGER-AUDIT.md.</t>
+          <t xml:space="preserve">A0 is VR-throttled: rocm-smi reports 1100 MHz, a sysfs sample under sustained load read 943 MHz. Its Hardware MFU column is therefore not a measure of efficiency.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every value re-derived from the raw ledgers. Where a published document disagreed, the ledger wins and the note says so. See LEDGER-AUDIT.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t xml:space="preserve">4</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t xml:space="preserve">Rows [3] were measured through the UNFIXED call path — tune_attention.py:529, t2_bringup.py:224/266, perfdq_diag.py:18 pass neither hip= nor scratch=; only the product path does.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" t="inlineStr">
+    <row r="58">
+      <c r="B58" t="inlineStr">
         <is>
           <t xml:space="preserve">Part of the 0.85 ms floor IS the per-call hipModuleLoad. Re-measuring the fixed path gives 8.13-8.68 ms (not 10.16), i.e. ~2.18x rather than 1.74x. The gate threshold is likely set too high and needs re-taking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ledger impl_note is unreliable: it is a string assigned from --impl before anything runs. The auditable field is asm_fwd; the SQNR fingerprint (dk 50.61 / dv 50.83 vs the fused path's 52.31 / 52.71) is what proves the ASM backward ran.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ledger impl_note is unreliable: it is a string assigned from --impl before anything runs. The auditable field is asm_fwd; the SQNR fingerprint (dk 50.61 / dv 50.83 vs the fused path's 52.31 / 52.71) is what proves the ASM backward ran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t xml:space="preserve">6</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t xml:space="preserve">DO NOT quote MFU from any torchtitan log on this box: get_peak_flops() falls back to "assume A100" (312 TF/s) for an unrecognised device_name, and this box reports "AMD Radeon Graphics". The tflop/s column is correct; mfu is not. || Cross-check: B0 at full clock also measures torch.mm(NN) at just 112.98 tflop/s against 1190.07 for a naive Triton GEMM (10.5x) — same order as A0's 13x. The missing NN tuning library is not specific to the throttled box.</t>
         </is>

</xml_diff>

<commit_message>
docs(0916): put the 32-layer production number in front -- 5.85x
The weekly material led with the 8-layer 6.21x. The 32-layer result is the one that transfers
to a real training claim, and it now exists: 1,984 -> 11,608 tps, all 20 steps, step time
16.5 s -> 2.82 s, peak memory 88.32% against the unpatched run's 87.98%.

Both HTML and the xlsx now say explicitly that the 8-layer rows exist to make A/B affordable
and must not be converted into a 32-layer claim -- a 32-layer step is four times the work per
token, so the two speedups describe different workloads even though they came from the same
patch.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
+++ b/output/0915__opt/mi455x-gfx1250-kernel-optimization.xlsx
@@ -17040,7 +17040,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:T60"/>
+  <dimension ref="A1:T61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.5"/>
@@ -18556,195 +18556,225 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t xml:space="preserve">32-LAYER PRODUCTION config (b=4 s=8192, 20 steps)</t>
+        </is>
+      </c>
+      <c r="B45">
+        <v>11608.0</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">steady jitter &lt;0.4%</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n=1 run, 13 steady steps</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.85x vs unpatched 1,984 (6.25x vs 1,858). Step 16.5s -&gt; 2.82s. Peak memory 88.32% vs unpatched 87.98%. THIS is the number to quote -- the 8-layer rows exist to make A/B affordable and are not comparable to a 32-layer result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t xml:space="preserve">ASM bwd ON / OFF (no workaround)</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t xml:space="preserve">6110.8 / 6128.1</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t xml:space="preserve">3.88% / 3.91%</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t xml:space="preserve">-0.28%, 0.15x sem — not significant; hence ASM bwd defaults OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[5] A0 — where a step goes (8 layers, step-10 torch profile, 5.2 s step)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">module</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ms</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">share</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">[5] A0 — where a step goes (8 layers, step-10 torch profile, 5.2 s step)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">hipBLASLt GEMM</t>
-        </is>
-      </c>
-      <c r="B49">
-        <v>4877.0</v>
+          <t xml:space="preserve">module</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ms</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">94%</t>
+          <t xml:space="preserve">share</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">4727 ms of it (97%) on MT32x16x32 — the wrong solution</t>
+          <t xml:space="preserve">note</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">attention (fwd+bwd)</t>
+          <t xml:space="preserve">hipBLASLt GEMM</t>
         </is>
       </c>
       <c r="B50">
-        <v>171.0</v>
+        <v>4877.0</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3%</t>
+          <t xml:space="preserve">94%</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">bwd_kernel_causal 138.55 + attn_fwd 32.09</t>
+          <t xml:space="preserve">4727 ms of it (97%) on MT32x16x32 — the wrong solution</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t xml:space="preserve">attention (fwd+bwd)</t>
+        </is>
+      </c>
+      <c r="B51">
+        <v>171.0</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.3%</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bwd_kernel_causal 138.55 + attn_fwd 32.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t xml:space="preserve">everything else</t>
         </is>
       </c>
-      <c r="B51">
+      <c r="B52">
         <v>140.0</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t xml:space="preserve">2.7%</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t xml:space="preserve">elementwise / optimizer / reduce / softmax</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOTES</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clocks differ ~2x between the two machines. Absolute values are NOT comparable across machines; no clock conversion is applied anywhere in this sheet.</t>
+          <t xml:space="preserve">NOTES</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">A0 is VR-throttled: rocm-smi reports 1100 MHz, a sysfs sample under sustained load read 943 MHz. Its Hardware MFU column is therefore not a measure of efficiency.</t>
+          <t xml:space="preserve">Clocks differ ~2x between the two machines. Absolute values are NOT comparable across machines; no clock conversion is applied anywhere in this sheet.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every value re-derived from the raw ledgers. Where a published document disagreed, the ledger wins and the note says so. See LEDGER-AUDIT.md.</t>
+          <t xml:space="preserve">A0 is VR-throttled: rocm-smi reports 1100 MHz, a sysfs sample under sustained load read 943 MHz. Its Hardware MFU column is therefore not a measure of efficiency.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every value re-derived from the raw ledgers. Where a published document disagreed, the ledger wins and the note says so. See LEDGER-AUDIT.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t xml:space="preserve">4</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t xml:space="preserve">Rows [3] were measured through the UNFIXED call path — tune_attention.py:529, t2_bringup.py:224/266, perfdq_diag.py:18 pass neither hip= nor scratch=; only the product path does.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" t="inlineStr">
+    <row r="59">
+      <c r="B59" t="inlineStr">
         <is>
           <t xml:space="preserve">Part of the 0.85 ms floor IS the per-call hipModuleLoad. Re-measuring the fixed path gives 8.13-8.68 ms (not 10.16), i.e. ~2.18x rather than 1.74x. The gate threshold is likely set too high and needs re-taking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ledger impl_note is unreliable: it is a string assigned from --impl before anything runs. The auditable field is asm_fwd; the SQNR fingerprint (dk 50.61 / dv 50.83 vs the fused path's 52.31 / 52.71) is what proves the ASM backward ran.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ledger impl_note is unreliable: it is a string assigned from --impl before anything runs. The auditable field is asm_fwd; the SQNR fingerprint (dk 50.61 / dv 50.83 vs the fused path's 52.31 / 52.71) is what proves the ASM backward ran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t xml:space="preserve">6</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t xml:space="preserve">DO NOT quote MFU from any torchtitan log on this box: get_peak_flops() falls back to "assume A100" (312 TF/s) for an unrecognised device_name, and this box reports "AMD Radeon Graphics". The tflop/s column is correct; mfu is not. || Cross-check: B0 at full clock also measures torch.mm(NN) at just 112.98 tflop/s against 1190.07 for a naive Triton GEMM (10.5x) — same order as A0's 13x. The missing NN tuning library is not specific to the throttled box.</t>
         </is>

</xml_diff>